<commit_message>
Add points for 7mw80b82sfqh1le7swr7l8zdg_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/7mw80b82sfqh1le7swr7l8zdg_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/7mw80b82sfqh1le7swr7l8zdg_playerlog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG23"/>
+  <dimension ref="A1:BG33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -780,14 +780,14 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -819,7 +819,7 @@
         <v>1</v>
       </c>
       <c r="AE2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF2" t="n">
         <v>0</v>
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
@@ -862,7 +862,7 @@
         <v>0</v>
       </c>
       <c r="AV2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -951,14 +951,14 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -990,10 +990,10 @@
         <v>1</v>
       </c>
       <c r="AE3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF3" t="n">
-        <v>-0</v>
+        <v>-0.4</v>
       </c>
       <c r="AG3" t="n">
         <v>1</v>
@@ -1004,21 +1004,21 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>0.33571589</v>
+        <v>-0.07900053000000004</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>+0.04</t>
+          <t>-0.48</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="AL3" t="n">
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN3" t="n">
         <v>0</v>
@@ -1033,16 +1033,16 @@
         <v>1</v>
       </c>
       <c r="AR3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AT3" t="n">
         <v>0</v>
       </c>
       <c r="AU3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AV3" t="n">
         <v>0</v>
@@ -1120,10 +1120,12 @@
           <t>9klc6ewu3oumq8eh96vr307pw</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K4" t="inlineStr"/>
@@ -1134,14 +1136,14 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1149,7 +1151,7 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
@@ -1173,13 +1175,13 @@
         <v>1</v>
       </c>
       <c r="AE4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF4" t="n">
-        <v>-0</v>
+        <v>-0.4</v>
       </c>
       <c r="AG4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
@@ -1187,21 +1189,21 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>0.6417859</v>
+        <v>0.33320987</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>+0.34</t>
+          <t>-0.07</t>
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="AL4" t="n">
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
@@ -1213,19 +1215,19 @@
         <v>1</v>
       </c>
       <c r="AQ4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AS4" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="AT4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="AV4" t="n">
         <v>0</v>
@@ -1256,7 +1258,7 @@
         <v>0</v>
       </c>
       <c r="BF4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BG4" t="n">
         <v>0</v>
@@ -1303,10 +1305,12 @@
           <t>9dvabsnjupk6spntn81200lqs</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
@@ -1317,14 +1321,14 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1332,7 +1336,7 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
@@ -1356,13 +1360,13 @@
         <v>1</v>
       </c>
       <c r="AE5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF5" t="n">
-        <v>-0</v>
+        <v>-0.4</v>
       </c>
       <c r="AG5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
@@ -1370,21 +1374,21 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>0.15122118</v>
+        <v>-0.4738700500000001</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>-0.88</t>
         </is>
       </c>
       <c r="AK5" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
       </c>
       <c r="AM5" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="AN5" t="n">
         <v>0</v>
@@ -1399,17 +1403,17 @@
         <v>0</v>
       </c>
       <c r="AR5" t="n">
+        <v>4</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>6</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU5" t="n">
         <v>3</v>
       </c>
-      <c r="AS5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU5" t="n">
-        <v>2</v>
-      </c>
       <c r="AV5" t="n">
         <v>1</v>
       </c>
@@ -1417,7 +1421,7 @@
         <v>0</v>
       </c>
       <c r="AX5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY5" t="n">
         <v>0</v>
@@ -1500,14 +1504,14 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1515,7 +1519,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -1539,10 +1543,10 @@
         <v>1</v>
       </c>
       <c r="AE6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF6" t="n">
-        <v>-0</v>
+        <v>-0.4</v>
       </c>
       <c r="AG6" t="n">
         <v>1</v>
@@ -1553,21 +1557,21 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>0.05127147999999998</v>
+        <v>0.12953815</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>-0.25</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="AK6" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="AL6" t="n">
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN6" t="n">
         <v>0</v>
@@ -1579,22 +1583,22 @@
         <v>0</v>
       </c>
       <c r="AQ6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AS6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AT6" t="n">
         <v>1</v>
       </c>
       <c r="AU6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW6" t="n">
         <v>0</v>
@@ -1622,7 +1626,7 @@
         <v>0</v>
       </c>
       <c r="BF6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG6" t="n">
         <v>0</v>
@@ -1683,14 +1687,14 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1698,7 +1702,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
@@ -1722,10 +1726,10 @@
         <v>1</v>
       </c>
       <c r="AE7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF7" t="n">
-        <v>-0</v>
+        <v>-0.4</v>
       </c>
       <c r="AG7" t="n">
         <v>1</v>
@@ -1736,48 +1740,48 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0.6617481200000001</v>
+        <v>0.28151987</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>+0.36</t>
+          <t>-0.12</t>
         </is>
       </c>
       <c r="AK7" t="n">
+        <v>17</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>97</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>8</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU7" t="n">
         <v>3</v>
       </c>
-      <c r="AL7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>50</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS7" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU7" t="n">
-        <v>1</v>
-      </c>
       <c r="AV7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW7" t="n">
         <v>0</v>
@@ -1866,14 +1870,14 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1881,7 +1885,7 @@
         </is>
       </c>
       <c r="S8" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
@@ -1905,10 +1909,10 @@
         <v>1</v>
       </c>
       <c r="AE8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF8" t="n">
-        <v>-0</v>
+        <v>-0.1</v>
       </c>
       <c r="AG8" t="n">
         <v>1</v>
@@ -1919,21 +1923,21 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>1.08303771</v>
+        <v>0.49564328</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>+0.78</t>
+          <t>+0.09</t>
         </is>
       </c>
       <c r="AK8" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="AL8" t="n">
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN8" t="n">
         <v>1</v>
@@ -1945,19 +1949,19 @@
         <v>0</v>
       </c>
       <c r="AQ8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR8" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU8" t="n">
         <v>3</v>
-      </c>
-      <c r="AS8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU8" t="n">
-        <v>2</v>
       </c>
       <c r="AV8" t="n">
         <v>0</v>
@@ -1988,7 +1992,7 @@
         <v>0</v>
       </c>
       <c r="BF8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BG8" t="n">
         <v>0</v>
@@ -2049,14 +2053,14 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -2064,7 +2068,7 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
@@ -2088,10 +2092,10 @@
         <v>1</v>
       </c>
       <c r="AE9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF9" t="n">
-        <v>-0</v>
+        <v>-0.1</v>
       </c>
       <c r="AG9" t="n">
         <v>1</v>
@@ -2102,21 +2106,21 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>0.06379616999999999</v>
+        <v>0.04455535999999993</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>-0.23</t>
+          <t>-0.36</t>
         </is>
       </c>
       <c r="AK9" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="AL9" t="n">
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN9" t="n">
         <v>0</v>
@@ -2128,10 +2132,10 @@
         <v>0</v>
       </c>
       <c r="AQ9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AR9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AS9" t="n">
         <v>2</v>
@@ -2140,10 +2144,10 @@
         <v>0</v>
       </c>
       <c r="AU9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AV9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW9" t="n">
         <v>0</v>
@@ -2171,7 +2175,7 @@
         <v>0</v>
       </c>
       <c r="BF9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BG9" t="n">
         <v>0</v>
@@ -2218,10 +2222,12 @@
           <t>a8pgjuz5yrbxyf1t905gj327d</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>2</v>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -2232,14 +2238,14 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -2247,7 +2253,7 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
@@ -2271,13 +2277,13 @@
         <v>1</v>
       </c>
       <c r="AE10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF10" t="n">
         <v>0</v>
       </c>
       <c r="AG10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
@@ -2285,21 +2291,21 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>0.98298167</v>
+        <v>0.8977095399999999</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>+0.68</t>
+          <t>+0.49</t>
         </is>
       </c>
       <c r="AK10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AL10" t="n">
         <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>50</v>
+        <v>83</v>
       </c>
       <c r="AN10" t="n">
         <v>0</v>
@@ -2311,10 +2317,10 @@
         <v>1</v>
       </c>
       <c r="AQ10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AR10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS10" t="n">
         <v>0</v>
@@ -2354,7 +2360,7 @@
         <v>0</v>
       </c>
       <c r="BF10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BG10" t="n">
         <v>0</v>
@@ -2401,10 +2407,12 @@
           <t>4iajf99dfecbzncfo65s0i0dm</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>2</v>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -2415,14 +2423,18 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>50</v>
-      </c>
-      <c r="O11" t="inlineStr"/>
+        <v>91</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>LAM(2)</t>
+        </is>
+      </c>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2430,10 +2442,16 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>50</v>
-      </c>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="inlineStr"/>
+        <v>76</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>LAM(2)</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>15</v>
+      </c>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
@@ -2454,13 +2472,13 @@
         <v>1</v>
       </c>
       <c r="AE11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AF11" t="n">
-        <v>-0</v>
+        <v>-0.1</v>
       </c>
       <c r="AG11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -2468,21 +2486,21 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.02077103</v>
+        <v>0.04869290000000007</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>-0.28</t>
+          <t>-0.35</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
       </c>
       <c r="AM11" t="n">
-        <v>50</v>
+        <v>91</v>
       </c>
       <c r="AN11" t="n">
         <v>0</v>
@@ -2491,13 +2509,13 @@
         <v>0</v>
       </c>
       <c r="AP11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AQ11" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="AR11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AS11" t="n">
         <v>0</v>
@@ -2506,7 +2524,7 @@
         <v>0</v>
       </c>
       <c r="AU11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV11" t="n">
         <v>0</v>
@@ -2537,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="BF11" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="BG11" t="n">
         <v>0</v>
@@ -2584,10 +2602,12 @@
           <t>eijd6yua2daogndd8o9br4n2t</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>2</v>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -2598,14 +2618,14 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2613,7 +2633,7 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
@@ -2637,13 +2657,13 @@
         <v>1</v>
       </c>
       <c r="AE12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF12" t="n">
-        <v>-0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
@@ -2651,21 +2671,21 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.04223183999999996</v>
+        <v>0.28250337</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>-0.26</t>
+          <t>-0.12</t>
         </is>
       </c>
       <c r="AK12" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="AL12" t="n">
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="AN12" t="n">
         <v>0</v>
@@ -2677,10 +2697,10 @@
         <v>1</v>
       </c>
       <c r="AQ12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS12" t="n">
         <v>0</v>
@@ -2695,7 +2715,7 @@
         <v>0</v>
       </c>
       <c r="AW12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX12" t="n">
         <v>0</v>
@@ -2720,7 +2740,7 @@
         <v>0</v>
       </c>
       <c r="BF12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="BG12" t="n">
         <v>0</v>
@@ -2734,37 +2754,37 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>L. Zidane</t>
+          <t>Mohammad Abu Hasheesh</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>23</t>
+          <t xml:space="preserve"> 2</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>LWB</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>aphehe8k4e6o0vho93xmxcyxh</t>
+          <t>bjo9f0df66c5ysu5pa8jehz4k</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -2773,30 +2793,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>84</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2</v>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="Q13" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>LWB</t>
         </is>
       </c>
       <c r="S13" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
@@ -2808,35 +2832,47 @@
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="AD13" t="n">
         <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF13" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>Mohammad Abu Hasheesh</t>
+        </is>
+      </c>
+      <c r="AI13" t="n">
+        <v>0.18806339</v>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>-0.22</t>
+        </is>
+      </c>
+      <c r="AK13" t="n">
+        <v>18</v>
+      </c>
       <c r="AL13" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
       <c r="AM13" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN13" t="n">
         <v>0</v>
@@ -2851,19 +2887,19 @@
         <v>0</v>
       </c>
       <c r="AR13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AS13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT13" t="n">
         <v>0</v>
       </c>
       <c r="AU13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AV13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AW13" t="n">
         <v>0</v>
@@ -2905,37 +2941,37 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>R. Belghali</t>
+          <t>Mohammad Abu Zraiq</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 17</t>
+          <t xml:space="preserve"> 7</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>RAM(2)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>88bb68l7u2rd453gz303p4qvo</t>
+          <t>9q6ef6upesu0oc8vhap6enomi</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -2944,33 +2980,47 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>91</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2</v>
+      </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N14" t="n">
-        <v>50</v>
-      </c>
-      <c r="O14" t="inlineStr"/>
+        <v>6</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>LAM(2)</t>
+        </is>
+      </c>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="Q14" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>RAM(2)</t>
         </is>
       </c>
       <c r="S14" t="n">
-        <v>50</v>
-      </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
+        <v>0.1</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>LAM(2)</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>5.9</v>
+      </c>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
@@ -2979,47 +3029,47 @@
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="AD14" t="n">
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF14" t="n">
-        <v>-0.2</v>
+        <v>-0</v>
       </c>
       <c r="AG14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>R. Belghali</t>
+          <t>Mohammad Abu Zraiq</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.002031999999999951</v>
+        <v>-0.05308202</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t>-0.46</t>
         </is>
       </c>
       <c r="AK14" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="AL14" t="n">
-        <v>0</v>
+        <v>91</v>
       </c>
       <c r="AM14" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN14" t="n">
         <v>0</v>
@@ -3031,7 +3081,7 @@
         <v>0</v>
       </c>
       <c r="AQ14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR14" t="n">
         <v>0</v>
@@ -3074,7 +3124,7 @@
         <v>0</v>
       </c>
       <c r="BF14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BG14" t="n">
         <v>0</v>
@@ -3088,37 +3138,37 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>R. Aït-Nouri</t>
+          <t>Odeh Fakhoury</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 15</t>
+          <t xml:space="preserve"> 11</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RAM(2)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>9jxhgh1vhc531ho0ez5alfazu</t>
+          <t>cpzl0b545pvfuqec7uaqyhpn8</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -3127,33 +3177,47 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>75</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2</v>
+      </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N15" t="n">
-        <v>50</v>
-      </c>
-      <c r="O15" t="inlineStr"/>
+        <v>22</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="Q15" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RAM(2)</t>
         </is>
       </c>
       <c r="S15" t="n">
-        <v>50</v>
-      </c>
-      <c r="T15" t="inlineStr"/>
-      <c r="U15" t="inlineStr"/>
+        <v>16.1</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="U15" t="n">
+        <v>5.9</v>
+      </c>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
@@ -3162,12 +3226,12 @@
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="AD15" t="n">
@@ -3177,18 +3241,18 @@
         <v>1</v>
       </c>
       <c r="AF15" t="n">
-        <v>-0.2</v>
+        <v>-0.05</v>
       </c>
       <c r="AG15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>R. Aït-Nouri</t>
+          <t>Odeh Fakhoury</t>
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>-0.05679712000000009</v>
+        <v>0.0383761</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
@@ -3196,13 +3260,13 @@
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="AL15" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="AM15" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN15" t="n">
         <v>0</v>
@@ -3214,19 +3278,19 @@
         <v>0</v>
       </c>
       <c r="AQ15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AR15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AS15" t="n">
         <v>0</v>
       </c>
       <c r="AT15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU15" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="AV15" t="n">
         <v>0</v>
@@ -3257,7 +3321,7 @@
         <v>0</v>
       </c>
       <c r="BF15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BG15" t="n">
         <v>0</v>
@@ -3271,37 +3335,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>R. Zerrouki</t>
+          <t>Saleem Obaid</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6</t>
+          <t xml:space="preserve"> 17</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>LCB(3)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>dc119ejc7lls2rd3ywigl2smi</t>
+          <t>ai1a4jh1la0msxejxvdzzgfe1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -3310,30 +3374,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>90</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2</v>
+      </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N16" t="n">
-        <v>50</v>
+        <v>7</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="Q16" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>LCB(3)</t>
         </is>
       </c>
       <c r="S16" t="n">
-        <v>50</v>
+        <v>7</v>
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
@@ -3345,47 +3413,47 @@
       <c r="AA16" t="inlineStr"/>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="AC16" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="AD16" t="n">
         <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF16" t="n">
-        <v>-0.05</v>
+        <v>-0</v>
       </c>
       <c r="AG16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>R. Zerrouki</t>
+          <t>Saleem Obaid</t>
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>-0.3723671100000001</v>
+        <v>0.01846212</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>-0.67</t>
+          <t>-0.38</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="AL16" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="AM16" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN16" t="n">
         <v>0</v>
@@ -3400,13 +3468,13 @@
         <v>0</v>
       </c>
       <c r="AR16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT16" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AU16" t="n">
         <v>1</v>
@@ -3418,7 +3486,7 @@
         <v>0</v>
       </c>
       <c r="AX16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY16" t="n">
         <v>0</v>
@@ -3454,37 +3522,37 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A. Mandi</t>
+          <t>Ali Azaizeh</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 2</t>
+          <t xml:space="preserve"> 24</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>7c2qwyzh82a45s25zmdahrd91</t>
+          <t>chtopu29kdz63m0vjrmjou1as</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -3493,33 +3561,47 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>83</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2</v>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>50</v>
-      </c>
-      <c r="O17" t="inlineStr"/>
+        <v>14</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>RAM(2)</t>
+        </is>
+      </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="Q17" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S17" t="n">
-        <v>50</v>
-      </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
+        <v>8.1</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>RAM(2)</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>5.9</v>
+      </c>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
@@ -3528,47 +3610,47 @@
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+          <t>btn8ibf55ovz7y252vdiprbip</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="AD17" t="n">
         <v>0</v>
       </c>
       <c r="AE17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF17" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="AG17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>A. Mandi</t>
+          <t>Ali Azaizeh</t>
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>-0.15909451</v>
+        <v>0.02708274999999999</v>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>-0.46</t>
+          <t>-0.38</t>
         </is>
       </c>
       <c r="AK17" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="AL17" t="n">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="AM17" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN17" t="n">
         <v>0</v>
@@ -3583,16 +3665,16 @@
         <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AS17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AT17" t="n">
         <v>0</v>
       </c>
       <c r="AU17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AV17" t="n">
         <v>0</v>
@@ -3642,17 +3724,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>R. Bensebaini</t>
+          <t>L. Zidane</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 21</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3662,12 +3744,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>dqrzogrwznyks6whhfhq748ut</t>
+          <t>aphehe8k4e6o0vho93xmxcyxh</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -3684,22 +3766,22 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="S18" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -3720,38 +3802,26 @@
         </is>
       </c>
       <c r="AD18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE18" t="n">
         <v>1</v>
       </c>
       <c r="AF18" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="AG18" t="n">
         <v>1</v>
       </c>
-      <c r="AH18" t="inlineStr">
-        <is>
-          <t>R. Bensebaini</t>
-        </is>
-      </c>
-      <c r="AI18" t="n">
-        <v>0.09647366000000002</v>
-      </c>
-      <c r="AJ18" t="inlineStr">
-        <is>
-          <t>-0.20</t>
-        </is>
-      </c>
-      <c r="AK18" t="n">
-        <v>12</v>
-      </c>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="n">
         <v>0</v>
       </c>
       <c r="AM18" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN18" t="n">
         <v>0</v>
@@ -3766,19 +3836,19 @@
         <v>0</v>
       </c>
       <c r="AR18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AS18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AT18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AW18" t="n">
         <v>0</v>
@@ -3825,17 +3895,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>R. Mahrez</t>
+          <t>R. Belghali</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 7</t>
+          <t xml:space="preserve"> 17</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3845,12 +3915,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>exiribcpg9vnuq9ekhlk74dlh</t>
+          <t>88bb68l7u2rd453gz303p4qvo</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -3867,25 +3937,35 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>50</v>
-      </c>
-      <c r="O19" t="inlineStr"/>
+        <v>97</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>RWB</t>
+        </is>
+      </c>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="S19" t="n">
-        <v>50</v>
-      </c>
-      <c r="T19" t="inlineStr"/>
-      <c r="U19" t="inlineStr"/>
+        <v>85.2</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>RWB</t>
+        </is>
+      </c>
+      <c r="U19" t="n">
+        <v>11.8</v>
+      </c>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr"/>
@@ -3903,38 +3983,38 @@
         </is>
       </c>
       <c r="AD19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE19" t="n">
         <v>1</v>
       </c>
       <c r="AF19" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG19" t="n">
         <v>1</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>R. Mahrez</t>
+          <t>R. Belghali</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.53987313</v>
+        <v>0.41495004</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>+0.24</t>
+          <t>+0.01</t>
         </is>
       </c>
       <c r="AK19" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="AL19" t="n">
         <v>0</v>
       </c>
       <c r="AM19" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN19" t="n">
         <v>0</v>
@@ -3943,28 +4023,28 @@
         <v>0</v>
       </c>
       <c r="AP19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR19" t="n">
         <v>1</v>
       </c>
       <c r="AS19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT19" t="n">
         <v>0</v>
       </c>
       <c r="AU19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV19" t="n">
         <v>0</v>
       </c>
       <c r="AW19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX19" t="n">
         <v>0</v>
@@ -3989,7 +4069,7 @@
         <v>0</v>
       </c>
       <c r="BF19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BG19" t="n">
         <v>0</v>
@@ -4008,17 +4088,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>H. Boudaoui</t>
+          <t>R. Aït-Nouri</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 14</t>
+          <t xml:space="preserve"> 15</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4028,18 +4108,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>e7e68wlpiqqohpg71oh4vrbl6</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
+          <t>9jxhgh1vhc531ho0ez5alfazu</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>2</v>
+      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -4050,22 +4132,22 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="S20" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
@@ -4086,38 +4168,38 @@
         </is>
       </c>
       <c r="AD20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE20" t="n">
         <v>1</v>
       </c>
       <c r="AF20" t="n">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="AG20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>H. Boudaoui</t>
+          <t>R. Aït-Nouri</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.6219603699999999</v>
+        <v>0.30689543</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>+0.32</t>
+          <t>-0.10</t>
         </is>
       </c>
       <c r="AK20" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="AL20" t="n">
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="AN20" t="n">
         <v>0</v>
@@ -4126,22 +4208,22 @@
         <v>0</v>
       </c>
       <c r="AP20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AS20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT20" t="n">
         <v>1</v>
       </c>
       <c r="AU20" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="AV20" t="n">
         <v>0</v>
@@ -4172,7 +4254,7 @@
         <v>0</v>
       </c>
       <c r="BF20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BG20" t="n">
         <v>0</v>
@@ -4191,17 +4273,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>A. Gouiri</t>
+          <t>R. Zerrouki</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 9</t>
+          <t xml:space="preserve"> 6</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4211,18 +4293,20 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>6u2ob6fv950r1qve8uejkq2uh</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr"/>
+          <t>dc119ejc7lls2rd3ywigl2smi</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>2</v>
+      </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
@@ -4233,22 +4317,22 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="S21" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
@@ -4275,32 +4359,32 @@
         <v>1</v>
       </c>
       <c r="AF21" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>A. Gouiri</t>
+          <t>R. Zerrouki</t>
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>0.5181913</v>
+        <v>-0.3816926500000001</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>+0.22</t>
+          <t>-0.79</t>
         </is>
       </c>
       <c r="AK21" t="n">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="AL21" t="n">
         <v>0</v>
       </c>
       <c r="AM21" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="AN21" t="n">
         <v>0</v>
@@ -4312,16 +4396,16 @@
         <v>0</v>
       </c>
       <c r="AQ21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AR21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT21" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AU21" t="n">
         <v>1</v>
@@ -4330,10 +4414,10 @@
         <v>0</v>
       </c>
       <c r="AW21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY21" t="n">
         <v>0</v>
@@ -4355,7 +4439,7 @@
         <v>0</v>
       </c>
       <c r="BF21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BG21" t="n">
         <v>0</v>
@@ -4374,17 +4458,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>I. Maza</t>
+          <t>A. Mandi</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 22</t>
+          <t xml:space="preserve"> 2</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4394,12 +4478,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>9x0s8mzjc9ey0q812sn3poums</t>
+          <t>7c2qwyzh82a45s25zmdahrd91</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -4416,25 +4500,35 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>50</v>
-      </c>
-      <c r="O22" t="inlineStr"/>
+        <v>97</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>CB(3)</t>
+        </is>
+      </c>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="S22" t="n">
-        <v>50</v>
-      </c>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
+        <v>85.2</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>CB(3)</t>
+        </is>
+      </c>
+      <c r="U22" t="n">
+        <v>11.8</v>
+      </c>
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr"/>
       <c r="X22" t="inlineStr"/>
@@ -4452,38 +4546,38 @@
         </is>
       </c>
       <c r="AD22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE22" t="n">
         <v>1</v>
       </c>
       <c r="AF22" t="n">
-        <v>-0.05</v>
+        <v>-0.2</v>
       </c>
       <c r="AG22" t="n">
         <v>1</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>I. Maza</t>
+          <t>A. Mandi</t>
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>0.49587763</v>
+        <v>0.1231221599999999</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>+0.20</t>
+          <t>-0.28</t>
         </is>
       </c>
       <c r="AK22" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="AL22" t="n">
         <v>0</v>
       </c>
       <c r="AM22" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -4492,22 +4586,22 @@
         <v>0</v>
       </c>
       <c r="AP22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AQ22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AR22" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AS22" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AT22" t="n">
         <v>0</v>
       </c>
       <c r="AU22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AV22" t="n">
         <v>0</v>
@@ -4538,7 +4632,7 @@
         <v>0</v>
       </c>
       <c r="BF22" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="BG22" t="n">
         <v>0</v>
@@ -4557,17 +4651,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>F. Chaïbi</t>
+          <t>R. Bensebaini</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 10</t>
+          <t xml:space="preserve"> 21</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4577,12 +4671,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>684cguhktvth28ql6qgvvmcyc</t>
+          <t>dqrzogrwznyks6whhfhq748ut</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
@@ -4599,25 +4693,35 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>50</v>
-      </c>
-      <c r="O23" t="inlineStr"/>
+        <v>97</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>LCB(3)</t>
+        </is>
+      </c>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="S23" t="n">
-        <v>50</v>
-      </c>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
+        <v>85.2</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>LCB(3)</t>
+        </is>
+      </c>
+      <c r="U23" t="n">
+        <v>11.8</v>
+      </c>
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
@@ -4635,38 +4739,38 @@
         </is>
       </c>
       <c r="AD23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE23" t="n">
         <v>1</v>
       </c>
       <c r="AF23" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="AG23" t="n">
         <v>1</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>F. Chaïbi</t>
+          <t>R. Bensebaini</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.36206755</v>
+        <v>0.75096178</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>+0.06</t>
+          <t>+0.35</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AL23" t="n">
         <v>0</v>
       </c>
       <c r="AM23" t="n">
-        <v>50</v>
+        <v>97</v>
       </c>
       <c r="AN23" t="n">
         <v>0</v>
@@ -4675,22 +4779,22 @@
         <v>0</v>
       </c>
       <c r="AP23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR23" t="n">
+        <v>7</v>
+      </c>
+      <c r="AS23" t="n">
         <v>4</v>
       </c>
-      <c r="AS23" t="n">
-        <v>0</v>
-      </c>
       <c r="AT23" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AU23" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AV23" t="n">
         <v>0</v>
@@ -4724,6 +4828,1938 @@
         <v>1</v>
       </c>
       <c r="BG23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>7mw80b82sfqh1le7swr7l8zdg</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>R. Mahrez</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 7</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>exiribcpg9vnuq9ekhlk74dlh</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>75</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>75</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="S24" t="n">
+        <v>75</v>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="AD24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>R. Mahrez</t>
+        </is>
+      </c>
+      <c r="AI24" t="n">
+        <v>1.71664394</v>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>+1.31</t>
+        </is>
+      </c>
+      <c r="AK24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>75</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>4</v>
+      </c>
+      <c r="AR24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD24" t="inlineStr"/>
+      <c r="BE24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF24" t="n">
+        <v>8</v>
+      </c>
+      <c r="BG24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>7mw80b82sfqh1le7swr7l8zdg</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>H. Boudaoui</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 14</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>e7e68wlpiqqohpg71oh4vrbl6</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>45</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>45</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="S25" t="n">
+        <v>45</v>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="AD25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>H. Boudaoui</t>
+        </is>
+      </c>
+      <c r="AI25" t="n">
+        <v>0.63987049</v>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>+0.24</t>
+        </is>
+      </c>
+      <c r="AK25" t="n">
+        <v>8</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>90</v>
+      </c>
+      <c r="AN25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD25" t="inlineStr"/>
+      <c r="BE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>7mw80b82sfqh1le7swr7l8zdg</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>A. Gouiri</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 9</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>6u2ob6fv950r1qve8uejkq2uh</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>2</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>85</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>85</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S26" t="n">
+        <v>45</v>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="U26" t="n">
+        <v>40</v>
+      </c>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="AD26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>A. Gouiri</t>
+        </is>
+      </c>
+      <c r="AI26" t="n">
+        <v>1.60138096</v>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>+1.20</t>
+        </is>
+      </c>
+      <c r="AK26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>85</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD26" t="inlineStr"/>
+      <c r="BE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF26" t="n">
+        <v>5</v>
+      </c>
+      <c r="BG26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>7mw80b82sfqh1le7swr7l8zdg</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>I. Maza</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 22</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>9x0s8mzjc9ey0q812sn3poums</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>97</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>LAM(2)</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>97</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>LAM(2)</t>
+        </is>
+      </c>
+      <c r="U27" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="AD27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>I. Maza</t>
+        </is>
+      </c>
+      <c r="AI27" t="n">
+        <v>2.03962255</v>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>+1.64</t>
+        </is>
+      </c>
+      <c r="AK27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>97</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>8</v>
+      </c>
+      <c r="AR27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD27" t="inlineStr"/>
+      <c r="BE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF27" t="n">
+        <v>12</v>
+      </c>
+      <c r="BG27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>7mw80b82sfqh1le7swr7l8zdg</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>F. Chaïbi</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 10</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>684cguhktvth28ql6qgvvmcyc</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>97</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>LCM(2), LDM(2)</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>97</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="S28" t="n">
+        <v>45</v>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
+      <c r="U28" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>LDM(2)</t>
+        </is>
+      </c>
+      <c r="W28" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="AD28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>F. Chaïbi</t>
+        </is>
+      </c>
+      <c r="AI28" t="n">
+        <v>0.6645577</v>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>+0.26</t>
+        </is>
+      </c>
+      <c r="AK28" t="n">
+        <v>7</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>97</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR28" t="n">
+        <v>9</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD28" t="inlineStr"/>
+      <c r="BE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF28" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>7mw80b82sfqh1le7swr7l8zdg</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Z. Belaïd</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 5</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ua8idum4ugeq704np5of7azu</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>85</v>
+      </c>
+      <c r="L29" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>12</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>RCB(3)</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>85</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>97</v>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S29" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>RCB(3)</t>
+        </is>
+      </c>
+      <c r="U29" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="AD29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH29" t="inlineStr">
+        <is>
+          <t>Z. Belaïd</t>
+        </is>
+      </c>
+      <c r="AI29" t="n">
+        <v>0.5245562500000001</v>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>+0.12</t>
+        </is>
+      </c>
+      <c r="AK29" t="n">
+        <v>9</v>
+      </c>
+      <c r="AL29" t="n">
+        <v>85</v>
+      </c>
+      <c r="AM29" t="n">
+        <v>97</v>
+      </c>
+      <c r="AN29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS29" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU29" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD29" t="inlineStr"/>
+      <c r="BE29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF29" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>7mw80b82sfqh1le7swr7l8zdg</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>A. Hadj Moussa</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>dwyl0yii553i57u7azfa7d15g</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>75</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N30" t="n">
+        <v>22</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>RAM(2)</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>97</v>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="S30" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>RAM(2)</t>
+        </is>
+      </c>
+      <c r="U30" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="AD30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH30" t="inlineStr">
+        <is>
+          <t>A. Hadj Moussa</t>
+        </is>
+      </c>
+      <c r="AI30" t="n">
+        <v>0.3913421499999999</v>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="AK30" t="n">
+        <v>12</v>
+      </c>
+      <c r="AL30" t="n">
+        <v>75</v>
+      </c>
+      <c r="AM30" t="n">
+        <v>97</v>
+      </c>
+      <c r="AN30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ30" t="n">
+        <v>5</v>
+      </c>
+      <c r="AR30" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT30" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD30" t="inlineStr"/>
+      <c r="BE30" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF30" t="n">
+        <v>7</v>
+      </c>
+      <c r="BG30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>7mw80b82sfqh1le7swr7l8zdg</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>N. Benbouali</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 12</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>8o0a3k1bbim9y2kd6ljyoiwpg</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>45</v>
+      </c>
+      <c r="L31" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>52</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>97</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S31" t="n">
+        <v>52</v>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="inlineStr"/>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr"/>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="AD31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH31" t="inlineStr">
+        <is>
+          <t>N. Benbouali</t>
+        </is>
+      </c>
+      <c r="AI31" t="n">
+        <v>1.54014453</v>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>+1.14</t>
+        </is>
+      </c>
+      <c r="AK31" t="n">
+        <v>4</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>90</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>97</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AX31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD31" t="inlineStr"/>
+      <c r="BE31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>7mw80b82sfqh1le7swr7l8zdg</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>J. Hadjam</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 13</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>dzh403ofb9zatvornq0svb0gk</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>84</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>13</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>LWB</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>84</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>97</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>LB</t>
+        </is>
+      </c>
+      <c r="S32" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>LWB</t>
+        </is>
+      </c>
+      <c r="U32" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="AD32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>J. Hadjam</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>-0.003097899999999987</v>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>-0.41</t>
+        </is>
+      </c>
+      <c r="AK32" t="n">
+        <v>26</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>84</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>97</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD32" t="inlineStr"/>
+      <c r="BE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF32" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>7mw80b82sfqh1le7swr7l8zdg</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>N. Bentaleb</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 19</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>6ynchgp6o4tajwvnfdnoo11at</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>45</v>
+      </c>
+      <c r="L33" t="n">
+        <v>2</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>52</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>RDM(2)</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>97</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>RDM(2)</t>
+        </is>
+      </c>
+      <c r="U33" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>cbx8lz7loz866tsoawwrpxyl9</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>Algeria</t>
+        </is>
+      </c>
+      <c r="AD33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>N. Bentaleb</t>
+        </is>
+      </c>
+      <c r="AI33" t="n">
+        <v>0.35157374</v>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>-0.05</t>
+        </is>
+      </c>
+      <c r="AK33" t="n">
+        <v>13</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>90</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>97</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD33" t="inlineStr"/>
+      <c r="BE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF33" t="n">
+        <v>3</v>
+      </c>
+      <c r="BG33" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>